<commit_message>
chore: run build script for workflow profile
</commit_message>
<xml_diff>
--- a/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
@@ -16,16 +16,16 @@
     <sheet sheetId="10" name="@type=PropertyValue" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="@type=ItemList" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="@type=LearningResource" state="visible" r:id="rId15"/>
-    <sheet sheetId="13" name="@type=DigitalFormat" state="visible" r:id="rId16"/>
-    <sheet sheetId="14" name="@type=ComputerLanguage" state="visible" r:id="rId17"/>
-    <sheet sheetId="15" name="@type=DefinedTerm" state="visible" r:id="rId18"/>
+    <sheet sheetId="13" name="@type=DefinedTerm" state="visible" r:id="rId16"/>
+    <sheet sheetId="14" name="@type=DigitalFormat" state="visible" r:id="rId17"/>
+    <sheet sheetId="15" name="@type=ComputerLanguage" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="290">
   <si>
     <t>Name</t>
   </si>
@@ -165,7 +165,7 @@
     <t>"https://w3id.org/ro/workflow-crate/"</t>
   </si>
   <si>
-    <t>2026-07-22T15:33:37+10:00</t>
+    <t>2026-08-13T17:07:40+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
@@ -177,6 +177,21 @@
     <t/>
   </si>
   <si>
+    <t>crate-o-mode.json</t>
+  </si>
+  <si>
+    <t>Crate-O Editor Mode File</t>
+  </si>
+  <si>
+    <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/817", application/json]</t>
+  </si>
+  <si>
+    <t>2026-08-13T15:49:27+02:00</t>
+  </si>
+  <si>
+    <t>Mini Crate-O mode file for this profile (metadata, input groups, lookup and enabled classes — the schema/grammar is provided by the MASP profile crate itself).</t>
+  </si>
+  <si>
     <t>example_workflow.cwl</t>
   </si>
   <si>
@@ -204,21 +219,6 @@
     <t>text/markdown</t>
   </si>
   <si>
-    <t>crate-o-mode.json</t>
-  </si>
-  <si>
-    <t>Crate-O Editor Mode File</t>
-  </si>
-  <si>
-    <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/817", application/json]</t>
-  </si>
-  <si>
-    <t>2026-05-22T08:29:17+10:00</t>
-  </si>
-  <si>
-    <t>Mini Crate-O mode file for this profile (metadata, input groups, lookup and enabled classes — the schema/grammar is provided by the MASP profile crate itself).</t>
-  </si>
-  <si>
     <t>#author</t>
   </si>
   <si>
@@ -384,7 +384,7 @@
     <t>Main Workflow</t>
   </si>
   <si>
-    <t>["http://schema.org/MediaObject", "http://schema.org/SoftwareSourceCode", "https://bioschemas.org/ComputationalWorkflow"]</t>
+    <t>["http://schema.org/MediaObject", "http://schema.org/SoftwareSourceCode", "https://bioschemas.org/terms/ComputationalWorkflow"]</t>
   </si>
   <si>
     <t>The Main Workflow is the primary workflow of the RO-Crate. It represents the computational process that is described by the RO-Crate.</t>
@@ -450,7 +450,7 @@
     <t>Profile</t>
   </si>
   <si>
-    <t>["http://schema.org/CreativeWork", "http://schema.org/Profile"]</t>
+    <t>["http://schema.org/CreativeWork", "http://www.w3.org/ns/dx/prof/Profile"]</t>
   </si>
   <si>
     <t>A generic profile entity.</t>
@@ -696,10 +696,10 @@
     <t>#propertyValue_RO-Crate_Metadata_Descriptor.id</t>
   </si>
   <si>
-    <t>RO-Crate Metadadata Descriptor Identifier Constraint</t>
-  </si>
-  <si>
-    <t>Allowed identifier value constraint for RO-Crate Metadadata Descriptor.</t>
+    <t>RO-Crate Metadata Descriptor Identifier Constraint</t>
+  </si>
+  <si>
+    <t>Allowed identifier value constraint for RO-Crate Metadata Descriptor.</t>
   </si>
   <si>
     <t>ro-crate-metadata.json</t>
@@ -765,6 +765,18 @@
     <t>["https://w3id.org/workflowhub/workflow-ro-crate#cwl", "https://w3id.org/workflowhub/workflow-ro-crate#galaxy", "https://w3id.org/workflowhub/workflow-ro-crate#knime", "https://w3id.org/workflowhub/workflow-ro-crate#nextflow", "https://w3id.org/workflowhub/workflow-ro-crate#snakemake"]</t>
   </si>
   <si>
+    <t>#conformanceIndicators</t>
+  </si>
+  <si>
+    <t>Supported conformsTo identifiers</t>
+  </si>
+  <si>
+    <t>Canonical identifiers that indicate conformance to this profile.</t>
+  </si>
+  <si>
+    <t>"https://w3id.org/ro/workflow-crate/1.0"</t>
+  </si>
+  <si>
     <t>#programmingLanguageCWLList</t>
   </si>
   <si>
@@ -774,18 +786,6 @@
     <t>A list containing only the Common Workflow Language (CWL) as a programming language for the Workflow Description.</t>
   </si>
   <si>
-    <t>#conformanceIndicators</t>
-  </si>
-  <si>
-    <t>Supported conformsTo identifiers</t>
-  </si>
-  <si>
-    <t>Canonical identifiers that indicate conformance to this profile.</t>
-  </si>
-  <si>
-    <t>"https://w3id.org/ro/workflow-crate/1.0"</t>
-  </si>
-  <si>
     <t>#WorkflowExample</t>
   </si>
   <si>
@@ -798,12 +798,36 @@
     <t>["./", "https://w3id.org/workflowhub/workflow-ro-crate/1.0", "example_workflow.cwl", "diagram.svg", "README.md"]</t>
   </si>
   <si>
+    <t>https://w3id.org/ro/mode</t>
+  </si>
+  <si>
+    <t>DefinedTerm</t>
+  </si>
+  <si>
+    <t>Editor Mode</t>
+  </si>
+  <si>
+    <t>Role indicating a resource is an editor configuration mode file.</t>
+  </si>
+  <si>
+    <t>https://w3id.org/ro/conformance-indicators</t>
+  </si>
+  <si>
+    <t>Role indicating a resource enumerates identifiers that are accepted as conformance indicators for the profile.</t>
+  </si>
+  <si>
+    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/471</t>
+  </si>
+  <si>
+    <t>DigitalFormat</t>
+  </si>
+  <si>
+    <t>Hypertext Markup Language</t>
+  </si>
+  <si>
     <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/1149</t>
   </si>
   <si>
-    <t>DigitalFormat</t>
-  </si>
-  <si>
     <t>Markdown</t>
   </si>
   <si>
@@ -813,12 +837,6 @@
     <t>JSON Data Interchange Format</t>
   </si>
   <si>
-    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/471</t>
-  </si>
-  <si>
-    <t>Hypertext Markup Language</t>
-  </si>
-  <si>
     <t>alternateName</t>
   </si>
   <si>
@@ -877,24 +895,6 @@
   </si>
   <si>
     <t>"https://snakemake.readthedocs.io"</t>
-  </si>
-  <si>
-    <t>https://w3id.org/ro/mode</t>
-  </si>
-  <si>
-    <t>DefinedTerm</t>
-  </si>
-  <si>
-    <t>Editor Mode</t>
-  </si>
-  <si>
-    <t>Role indicating a resource is an editor configuration mode file.</t>
-  </si>
-  <si>
-    <t>https://w3id.org/ro/conformance-indicators</t>
-  </si>
-  <si>
-    <t>Role indicating a resource enumerates identifiers that are accepted as conformance indicators for the profile.</t>
   </si>
 </sst>
 </file>
@@ -1494,7 +1494,7 @@
         <v>228</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1628,24 +1628,24 @@
         <v>248</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B5" t="s">
         <v>239</v>
       </c>
       <c r="C5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E5" t="s">
-        <v>252</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1704,6 +1704,62 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1723,35 +1779,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B2" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C2" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B3" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C3" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B4" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C4" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -1760,7 +1816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1779,10 +1835,10 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="E1" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="F1" t="s">
         <v>67</v>
@@ -1790,145 +1846,89 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D2" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="E2" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="F2" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B3" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C3" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="F3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B4" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C4" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="E4" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="F4" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C5" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E5" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="F5" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B6" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C6" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="E6" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="F6" t="s">
-        <v>283</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="4" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>284</v>
-      </c>
-      <c r="B2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D2" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>288</v>
-      </c>
-      <c r="B3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D3" t="s">
         <v>289</v>
       </c>
     </row>
@@ -2119,66 +2119,66 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>50</v>
       </c>
       <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
         <v>51</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s">
         <v>28</v>
       </c>
-      <c r="I4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+      <c r="C6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
       </c>
-      <c r="C7" t="s">
-        <v>60</v>
-      </c>
       <c r="D7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G7" t="s">
         <v>63</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2658,7 +2658,7 @@
         <v>141</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -2752,6 +2752,9 @@
       <c r="C3" t="s">
         <v>153</v>
       </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
       <c r="E3" t="s">
         <v>150</v>
       </c>
@@ -3044,6 +3047,9 @@
       </c>
       <c r="C13" t="s">
         <v>191</v>
+      </c>
+      <c r="D13" t="s">
+        <v>36</v>
       </c>
       <c r="E13" t="s">
         <v>184</v>

</xml_diff>

<commit_message>
chore: regenerate after merging main
</commit_message>
<xml_diff>
--- a/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="291">
   <si>
     <t>Name</t>
   </si>
@@ -165,13 +165,16 @@
     <t>"https://w3id.org/ro/workflow-crate/"</t>
   </si>
   <si>
-    <t>2026-08-13T17:20:36+02:00</t>
+    <t>2026-08-13T17:34:50+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
   </si>
   <si>
     <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/1149", text/markdown]</t>
+  </si>
+  <si>
+    <t>2026-08-13T17:34:57+02:00</t>
   </si>
   <si>
     <t/>
@@ -1402,30 +1405,30 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1436,19 +1439,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1459,19 +1462,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1482,19 +1485,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1505,19 +1508,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1528,19 +1531,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1577,75 +1580,75 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1681,19 +1684,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -1726,30 +1729,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -1779,35 +1782,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -1835,101 +1838,101 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2110,10 +2113,10 @@
         <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
         <v>45</v>
@@ -2121,61 +2124,61 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
         <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
@@ -2208,13 +2211,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2242,7 +2245,7 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
@@ -2253,47 +2256,47 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2321,115 +2324,115 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2457,16 +2460,16 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H1" t="s">
         <v>8</v>
@@ -2474,19 +2477,19 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2497,16 +2500,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -2515,64 +2518,64 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -2583,19 +2586,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -2606,19 +2609,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -2629,33 +2632,33 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -2664,7 +2667,7 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2692,45 +2695,45 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J1" t="s">
         <v>6</v>
       </c>
       <c r="K1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2739,24 +2742,24 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D3" t="s">
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -2765,10 +2768,10 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J3" t="s">
         <v>36</v>
@@ -2776,106 +2779,106 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J4" t="s">
         <v>8</v>
       </c>
       <c r="K4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J5" t="s">
         <v>24</v>
       </c>
       <c r="K5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J6" t="s">
         <v>16</v>
       </c>
       <c r="K6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -2884,10 +2887,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J7" t="s">
         <v>25</v>
@@ -2895,19 +2898,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D8" t="s">
         <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -2916,10 +2919,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J8" t="s">
         <v>39</v>
@@ -2927,19 +2930,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -2948,10 +2951,10 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J9" t="s">
         <v>39</v>
@@ -2959,25 +2962,25 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J10" t="s">
         <v>18</v>
@@ -2985,19 +2988,19 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D11" t="s">
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -3006,24 +3009,24 @@
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -3032,27 +3035,27 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I12" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D13" t="s">
         <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -3061,10 +3064,10 @@
         <v>1</v>
       </c>
       <c r="H13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J13" t="s">
         <v>36</v>
@@ -3072,19 +3075,19 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D14" t="s">
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -3093,24 +3096,24 @@
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -3119,24 +3122,24 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -3145,59 +3148,59 @@
         <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I16" t="s">
+        <v>202</v>
+      </c>
+      <c r="J16" t="s">
         <v>201</v>
-      </c>
-      <c r="J16" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J17" t="s">
         <v>6</v>
       </c>
       <c r="K17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D18" t="s">
         <v>40</v>
       </c>
       <c r="E18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -3206,10 +3209,10 @@
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J18" t="s">
         <v>40</v>
@@ -3217,22 +3220,22 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D19" t="s">
         <v>6</v>
       </c>
       <c r="E19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J19" t="s">
         <v>6</v>
@@ -3240,22 +3243,22 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B20" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J20" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
fix: invalid key casing in 5 rules
</commit_message>
<xml_diff>
--- a/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="289">
   <si>
     <t>Name</t>
   </si>
@@ -165,7 +165,7 @@
     <t>"https://w3id.org/ro/workflow-crate/"</t>
   </si>
   <si>
-    <t>2026-08-13T17:34:50+02:00</t>
+    <t>2026-08-13T17:35:11+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
@@ -174,9 +174,6 @@
     <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/1149", text/markdown]</t>
   </si>
   <si>
-    <t>2026-08-13T17:34:57+02:00</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -343,9 +340,6 @@
   </si>
   <si>
     <t>prov:specializationOf</t>
-  </si>
-  <si>
-    <t>Description</t>
   </si>
   <si>
     <t>sh:minCount</t>
@@ -1405,30 +1399,30 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" t="s">
         <v>214</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>215</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>216</v>
-      </c>
-      <c r="D2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E2" t="s">
-        <v>218</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1439,19 +1433,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" t="s">
         <v>219</v>
       </c>
-      <c r="B3" t="s">
-        <v>215</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>220</v>
-      </c>
-      <c r="D3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E3" t="s">
-        <v>222</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1462,19 +1456,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" t="s">
         <v>223</v>
       </c>
-      <c r="B4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>224</v>
-      </c>
-      <c r="D4" t="s">
-        <v>225</v>
-      </c>
-      <c r="E4" t="s">
-        <v>226</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1485,19 +1479,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D5" t="s">
         <v>227</v>
       </c>
-      <c r="B5" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" t="s">
-        <v>228</v>
-      </c>
-      <c r="D5" t="s">
-        <v>229</v>
-      </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1508,19 +1502,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D6" t="s">
         <v>230</v>
       </c>
-      <c r="B6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>231</v>
-      </c>
-      <c r="D6" t="s">
-        <v>232</v>
-      </c>
-      <c r="E6" t="s">
-        <v>233</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1531,19 +1525,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" t="s">
         <v>234</v>
       </c>
-      <c r="B7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>235</v>
-      </c>
-      <c r="D7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E7" t="s">
-        <v>237</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1580,75 +1574,75 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C2" t="s">
         <v>239</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>240</v>
       </c>
-      <c r="C2" t="s">
-        <v>241</v>
-      </c>
-      <c r="D2" t="s">
-        <v>242</v>
-      </c>
       <c r="E2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D3" t="s">
         <v>243</v>
       </c>
-      <c r="B3" t="s">
-        <v>240</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>244</v>
-      </c>
-      <c r="D3" t="s">
-        <v>245</v>
-      </c>
-      <c r="E3" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" t="s">
         <v>247</v>
       </c>
-      <c r="B4" t="s">
-        <v>240</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>248</v>
-      </c>
-      <c r="D4" t="s">
-        <v>249</v>
-      </c>
-      <c r="E4" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" t="s">
         <v>251</v>
       </c>
-      <c r="B5" t="s">
-        <v>240</v>
-      </c>
-      <c r="C5" t="s">
-        <v>252</v>
-      </c>
-      <c r="D5" t="s">
-        <v>253</v>
-      </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1684,19 +1678,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C2" t="s">
         <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -1729,30 +1723,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C2" t="s">
         <v>258</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>259</v>
-      </c>
-      <c r="C2" t="s">
-        <v>260</v>
-      </c>
-      <c r="D2" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -1782,35 +1776,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C2" t="s">
         <v>264</v>
-      </c>
-      <c r="B2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C2" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B4" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -1838,101 +1832,101 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" t="s">
         <v>273</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>274</v>
       </c>
-      <c r="C2" t="s">
-        <v>252</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>275</v>
-      </c>
-      <c r="E2" t="s">
-        <v>276</v>
-      </c>
-      <c r="F2" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E3" t="s">
         <v>278</v>
       </c>
-      <c r="B3" t="s">
-        <v>274</v>
-      </c>
-      <c r="C3" t="s">
-        <v>279</v>
-      </c>
-      <c r="E3" t="s">
-        <v>280</v>
-      </c>
       <c r="F3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B4" t="s">
+        <v>272</v>
+      </c>
+      <c r="C4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E4" t="s">
         <v>281</v>
       </c>
-      <c r="B4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C4" t="s">
-        <v>282</v>
-      </c>
-      <c r="E4" t="s">
-        <v>283</v>
-      </c>
       <c r="F4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>282</v>
+      </c>
+      <c r="B5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" t="s">
+        <v>283</v>
+      </c>
+      <c r="E5" t="s">
         <v>284</v>
       </c>
-      <c r="B5" t="s">
-        <v>274</v>
-      </c>
-      <c r="C5" t="s">
-        <v>285</v>
-      </c>
-      <c r="E5" t="s">
-        <v>286</v>
-      </c>
       <c r="F5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>285</v>
+      </c>
+      <c r="B6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E6" t="s">
         <v>287</v>
       </c>
-      <c r="B6" t="s">
-        <v>274</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>288</v>
-      </c>
-      <c r="E6" t="s">
-        <v>289</v>
-      </c>
-      <c r="F6" t="s">
-        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2113,10 +2107,10 @@
         <v>45</v>
       </c>
       <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
         <v>49</v>
-      </c>
-      <c r="G3" t="s">
-        <v>50</v>
       </c>
       <c r="H3" t="s">
         <v>45</v>
@@ -2124,61 +2118,61 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
         <v>42</v>
       </c>
       <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
         <v>52</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>53</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>54</v>
-      </c>
-      <c r="G4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
         <v>56</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
       </c>
       <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s">
         <v>58</v>
-      </c>
-      <c r="J5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
         <v>60</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>61</v>
-      </c>
-      <c r="C6" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
@@ -2211,13 +2205,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
         <v>65</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>66</v>
-      </c>
-      <c r="C2" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2245,7 +2239,7 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
@@ -2256,47 +2250,47 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
         <v>69</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>70</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>71</v>
-      </c>
-      <c r="D2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
         <v>73</v>
       </c>
-      <c r="B3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>74</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>75</v>
-      </c>
-      <c r="F3" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2324,115 +2318,115 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
         <v>80</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>81</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>82</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>83</v>
-      </c>
-      <c r="E2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" t="s">
         <v>85</v>
       </c>
-      <c r="B3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>86</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>87</v>
-      </c>
-      <c r="F3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
         <v>89</v>
       </c>
-      <c r="B4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>90</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>91</v>
-      </c>
-      <c r="F4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" t="s">
         <v>93</v>
       </c>
-      <c r="B5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>94</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>95</v>
-      </c>
-      <c r="F5" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
         <v>97</v>
       </c>
-      <c r="B6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>98</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>99</v>
-      </c>
-      <c r="F6" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
         <v>101</v>
       </c>
-      <c r="B7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>102</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>103</v>
-      </c>
-      <c r="F7" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2443,13 +2437,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="8" width="20" customWidth="1"/>
+    <col min="1" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2460,122 +2454,119 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
         <v>105</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>106</v>
-      </c>
-      <c r="F1" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
         <v>109</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>110</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>111</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>112</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" t="s">
         <v>113</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
         <v>114</v>
       </c>
-      <c r="B3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>115</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>116</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="B4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="D4" t="s">
         <v>118</v>
       </c>
-      <c r="B4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>119</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>120</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="B5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
         <v>122</v>
       </c>
-      <c r="B5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>123</v>
       </c>
-      <c r="D5" t="s">
-        <v>124</v>
-      </c>
       <c r="G5">
         <v>1</v>
-      </c>
-      <c r="H5" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" t="s">
         <v>126</v>
       </c>
-      <c r="B6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>127</v>
-      </c>
-      <c r="D6" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" t="s">
-        <v>129</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -2586,19 +2577,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" t="s">
         <v>130</v>
-      </c>
-      <c r="B7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" t="s">
-        <v>132</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -2609,19 +2600,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E8" t="s">
         <v>133</v>
-      </c>
-      <c r="B8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C8" t="s">
-        <v>134</v>
-      </c>
-      <c r="D8" t="s">
-        <v>116</v>
-      </c>
-      <c r="E8" t="s">
-        <v>135</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -2632,42 +2623,42 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D9" t="s">
         <v>136</v>
       </c>
-      <c r="B9" t="s">
-        <v>110</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
         <v>137</v>
       </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>138</v>
       </c>
-      <c r="E9" t="s">
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="D10" t="s">
         <v>140</v>
       </c>
-      <c r="B10" t="s">
-        <v>110</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>141</v>
-      </c>
-      <c r="D10" t="s">
-        <v>142</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
         <v>1</v>
-      </c>
-      <c r="H10" t="s">
-        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2695,45 +2686,45 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H1" t="s">
         <v>144</v>
       </c>
-      <c r="E1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F1" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" t="s">
-        <v>146</v>
-      </c>
       <c r="I1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J1" t="s">
         <v>6</v>
       </c>
       <c r="K1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" t="s">
         <v>148</v>
-      </c>
-      <c r="B2" t="s">
-        <v>149</v>
-      </c>
-      <c r="C2" t="s">
-        <v>150</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2742,24 +2733,24 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D3" t="s">
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -2768,10 +2759,10 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J3" t="s">
         <v>36</v>
@@ -2779,106 +2770,106 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="I4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J4" t="s">
         <v>8</v>
       </c>
       <c r="K4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J5" t="s">
         <v>24</v>
       </c>
       <c r="K5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J6" t="s">
         <v>16</v>
       </c>
       <c r="K6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -2887,10 +2878,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J7" t="s">
         <v>25</v>
@@ -2898,19 +2889,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D8" t="s">
         <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -2919,10 +2910,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="J8" t="s">
         <v>39</v>
@@ -2930,19 +2921,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -2951,10 +2942,10 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="I9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="J9" t="s">
         <v>39</v>
@@ -2962,25 +2953,25 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J10" t="s">
         <v>18</v>
@@ -2988,19 +2979,19 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B11" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C11" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D11" t="s">
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -3009,24 +3000,24 @@
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -3035,27 +3026,27 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="I12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B13" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D13" t="s">
         <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -3064,10 +3055,10 @@
         <v>1</v>
       </c>
       <c r="H13" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I13" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J13" t="s">
         <v>36</v>
@@ -3075,19 +3066,19 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D14" t="s">
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -3096,24 +3087,24 @@
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -3122,24 +3113,24 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>197</v>
+      </c>
+      <c r="B16" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D16" t="s">
         <v>199</v>
       </c>
-      <c r="B16" t="s">
-        <v>149</v>
-      </c>
-      <c r="C16" t="s">
-        <v>200</v>
-      </c>
-      <c r="D16" t="s">
-        <v>201</v>
-      </c>
       <c r="E16" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -3148,59 +3139,59 @@
         <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J16" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="I17" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J17" t="s">
         <v>6</v>
       </c>
       <c r="K17" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C18" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D18" t="s">
         <v>40</v>
       </c>
       <c r="E18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -3209,10 +3200,10 @@
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="I18" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J18" t="s">
         <v>40</v>
@@ -3220,22 +3211,22 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D19" t="s">
         <v>6</v>
       </c>
       <c r="E19" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J19" t="s">
         <v>6</v>
@@ -3243,22 +3234,22 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B20" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J20" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
fix: add #programmingLanguageCWLList to schema hasPart
</commit_message>
<xml_diff>
--- a/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/workflow/profile-crate/ro-crate-metadata.xlsx
@@ -165,7 +165,7 @@
     <t>"https://w3id.org/ro/workflow-crate/"</t>
   </si>
   <si>
-    <t>2026-08-13T17:35:11+02:00</t>
+    <t>2026-08-14T16:49:04+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
@@ -276,7 +276,7 @@
     <t>"http://www.w3.org/ns/dx/prof/role/schema"</t>
   </si>
   <si>
-    <t>["#RO-Crate_Metadata_Descriptor", "#Root_Data_Entity", "#Class_MainWorkflow", "#Class_MainWorkflow_Description", "#class_CreativeWork_README", "#class_Dataset_Test_Directory", "#class_Dataset_Examples_Directory", "#Class_ImageObject_Diagram", "#RO-Crate_Metadata_Descriptor.id", "#RO-Crate_Metadata_Descriptor.about", "#prop_description_Dataset", "#prop_datePublished_Dataset", "#prop_license_Dataset", "#Property_mainEntity_Workflow", "#Property_programmingLanguage_Workflow", "#Property_programmingLanguage_WorkflowDescription", "#prop_conformsTo_Root_Data_Entity", "#Root_Data_Entity_conformsTo_value", "#Root_Data_Entity_profile_itemList", "#property_CreativeWork_README.id", "#propertyValue_property_CreativeWork_README.id", "#property_CreativeWork_README.encodingFormat", "#property_CreativeWork_README.about", "#property_Dataset_Test_Directory.id", "#property_Dataset_Examples_Directory.id", "#Property_MainWorkflow_subjectOf", "http://schema.org/name", "#Property_MainWorkflow_image", "#classProfile", "#prop_name_classProfile", "#prop_version_classProfile", "#programmingLanguages", "#propertyValue_RO-Crate_Metadata_Descriptor.id", "#propertyValue_property_CreativeWork_README.encodingFormat", "#propertyValue_property_Dataset_Test_Directory.id", "#propertyValue_property_Dataset_Examples_Directory.id"]</t>
+    <t>["#RO-Crate_Metadata_Descriptor", "#Root_Data_Entity", "#Class_MainWorkflow", "#Class_MainWorkflow_Description", "#class_CreativeWork_README", "#class_Dataset_Test_Directory", "#class_Dataset_Examples_Directory", "#Class_ImageObject_Diagram", "#RO-Crate_Metadata_Descriptor.id", "#RO-Crate_Metadata_Descriptor.about", "#prop_description_Dataset", "#prop_datePublished_Dataset", "#prop_license_Dataset", "#Property_mainEntity_Workflow", "#Property_programmingLanguage_Workflow", "#Property_programmingLanguage_WorkflowDescription", "#prop_conformsTo_Root_Data_Entity", "#Root_Data_Entity_conformsTo_value", "#Root_Data_Entity_profile_itemList", "#property_CreativeWork_README.id", "#propertyValue_property_CreativeWork_README.id", "#property_CreativeWork_README.encodingFormat", "#property_CreativeWork_README.about", "#property_Dataset_Test_Directory.id", "#property_Dataset_Examples_Directory.id", "#Property_MainWorkflow_subjectOf", "http://schema.org/name", "#Property_MainWorkflow_image", "#classProfile", "#prop_name_classProfile", "#prop_version_classProfile", "#programmingLanguages", "#propertyValue_RO-Crate_Metadata_Descriptor.id", "#propertyValue_property_CreativeWork_README.encodingFormat", "#propertyValue_property_Dataset_Test_Directory.id", "#propertyValue_property_Dataset_Examples_Directory.id", "#programmingLanguageCWLList"]</t>
   </si>
   <si>
     <t>#hasExampleWorkflow</t>
@@ -762,6 +762,15 @@
     <t>["https://w3id.org/workflowhub/workflow-ro-crate#cwl", "https://w3id.org/workflowhub/workflow-ro-crate#galaxy", "https://w3id.org/workflowhub/workflow-ro-crate#knime", "https://w3id.org/workflowhub/workflow-ro-crate#nextflow", "https://w3id.org/workflowhub/workflow-ro-crate#snakemake"]</t>
   </si>
   <si>
+    <t>#programmingLanguageCWLList</t>
+  </si>
+  <si>
+    <t>Common Workflow Language</t>
+  </si>
+  <si>
+    <t>A list containing only the Common Workflow Language (CWL) as a programming language for the Workflow Description.</t>
+  </si>
+  <si>
     <t>#conformanceIndicators</t>
   </si>
   <si>
@@ -772,15 +781,6 @@
   </si>
   <si>
     <t>"https://w3id.org/ro/workflow-crate/1.0"</t>
-  </si>
-  <si>
-    <t>#programmingLanguageCWLList</t>
-  </si>
-  <si>
-    <t>Common Workflow Language</t>
-  </si>
-  <si>
-    <t>A list containing only the Common Workflow Language (CWL) as a programming language for the Workflow Description.</t>
   </si>
   <si>
     <t>#WorkflowExample</t>
@@ -1625,24 +1625,24 @@
         <v>247</v>
       </c>
       <c r="E4" t="s">
-        <v>248</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
         <v>238</v>
       </c>
       <c r="C5" t="s">
+        <v>249</v>
+      </c>
+      <c r="D5" t="s">
         <v>250</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>251</v>
-      </c>
-      <c r="E5" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1849,7 +1849,7 @@
         <v>272</v>
       </c>
       <c r="C2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D2" t="s">
         <v>273</v>

</xml_diff>